<commit_message>
APEX 37 : visual mastering Credit Risk Intelligence, JEV et TypeSafe dans chaque feuille, couche Blue Premium + TypeSafe sur tous les exports Excel, questions TypeSafe avancées
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DkwQ8QV1wk6UyfQvHD3u4J
</commit_message>
<xml_diff>
--- a/exemples_risk_intelligence/ECOBANK_Data_Export_2026-09-30.xlsx
+++ b/exemples_risk_intelligence/ECOBANK_Data_Export_2026-09-30.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="T5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Escalade contentieux</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
       </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="T16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="T28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="T31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="T34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="T40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">En cours</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="T65" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -5602,7 +5602,7 @@
       </c>
       <c r="T71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">En cours</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="T72" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -6358,7 +6358,7 @@
       </c>
       <c r="T81" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="T85" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="T97" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -10526,7 +10526,7 @@
       </c>
       <c r="T135" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -11852,7 +11852,7 @@
       </c>
       <c r="T152" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Escalade contentieux</t>
         </is>
       </c>
     </row>
@@ -12312,7 +12312,7 @@
       </c>
       <c r="T158" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -12394,7 +12394,7 @@
       </c>
       <c r="T159" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>
@@ -12476,7 +12476,7 @@
       </c>
       <c r="T160" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Promesse de règlement</t>
         </is>
       </c>
     </row>
@@ -13462,7 +13462,7 @@
       </c>
       <c r="T173" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">À faire</t>
+          <t xml:space="preserve">Revue analyste</t>
         </is>
       </c>
     </row>

</xml_diff>